<commit_message>
data wrangling + cv-folds + first model
</commit_message>
<xml_diff>
--- a/features.xlsx
+++ b/features.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakoberhard/Library/CloudStorage/GoogleDrive-jakanterh@gmail.com/My Drive/uni/python/TBA_project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C67B5BE3-3166-5E42-A5B2-2A783521C87F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D29E5851-0560-E84E-9C3A-10DD19C89B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="116">
   <si>
     <t>feature</t>
   </si>
@@ -181,15 +181,6 @@
     <t>station_related_history</t>
   </si>
   <si>
-    <t>group by station and give delay (mean)</t>
-  </si>
-  <si>
-    <t>group by station and give delay (sd)</t>
-  </si>
-  <si>
-    <t>group by station and give q90 quantile of delay</t>
-  </si>
-  <si>
     <t>see above only for specific day</t>
   </si>
   <si>
@@ -199,33 +190,6 @@
     <t>start / stopover / destination</t>
   </si>
   <si>
-    <t>hist_delay_avg_station * day</t>
-  </si>
-  <si>
-    <t>hist_delay_sd_station * day</t>
-  </si>
-  <si>
-    <t>hist_delay_q9_station * day</t>
-  </si>
-  <si>
-    <t>hist_delay_avg_station * hour</t>
-  </si>
-  <si>
-    <t>hist_delay_sd_station * hour</t>
-  </si>
-  <si>
-    <t>hist_delay_q9_station * hour</t>
-  </si>
-  <si>
-    <t>hist_delay_q9_station</t>
-  </si>
-  <si>
-    <t>hist_delay_sd_station</t>
-  </si>
-  <si>
-    <t>hist_delay_avg_station</t>
-  </si>
-  <si>
     <t>availability historical data</t>
   </si>
   <si>
@@ -235,9 +199,6 @@
     <t>not needed</t>
   </si>
   <si>
-    <t>? (@eddi)</t>
-  </si>
-  <si>
     <t>variable not needed</t>
   </si>
   <si>
@@ -389,6 +350,30 @@
   </si>
   <si>
     <t>eventuell feature bauen</t>
+  </si>
+  <si>
+    <t>hour</t>
+  </si>
+  <si>
+    <t>indicating time of the day</t>
+  </si>
+  <si>
+    <t>hist_delay_station_avg/sd/q90/count</t>
+  </si>
+  <si>
+    <t>hist_delay_station_day_avg/sd/q90/count</t>
+  </si>
+  <si>
+    <t>hist_delay_station_hour_avg/sd/q90/count</t>
+  </si>
+  <si>
+    <t>group by station and give delay (mean/sd/q90/count)</t>
+  </si>
+  <si>
+    <t>count is added as indicator data quality</t>
+  </si>
+  <si>
+    <t>canceled</t>
   </si>
 </sst>
 </file>
@@ -699,7 +684,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -728,6 +713,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1008,10 +994,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.6640625" customWidth="1"/>
     <col min="4" max="4" width="22.5" bestFit="1" customWidth="1"/>
@@ -1032,19 +1018,19 @@
         <v>1</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -1057,17 +1043,17 @@
       <c r="C2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="16" t="s">
-        <v>69</v>
+      <c r="D2" s="15" t="s">
+        <v>55</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H2" s="5"/>
     </row>
@@ -1082,15 +1068,15 @@
         <v>20</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="7" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -1104,10 +1090,10 @@
         <v>20</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -1123,17 +1109,17 @@
       <c r="C5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="H5" s="7"/>
     </row>
@@ -1148,68 +1134,64 @@
         <v>20</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="H6" s="7"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>49</v>
+        <v>115</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>74</v>
-      </c>
+      <c r="D7" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
       <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="23" t="s">
+      <c r="D8" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="23" t="s">
         <v>22</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>13</v>
@@ -1217,95 +1199,95 @@
       <c r="C9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E9" s="23" t="s">
         <v>22</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="H9" s="7"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="D10" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E10" s="23" t="s">
         <v>22</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="H10" s="7"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E11" s="23" t="s">
         <v>22</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="H11" s="7"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="23" t="s">
         <v>22</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="H12" s="7"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>15</v>
@@ -1313,47 +1295,47 @@
       <c r="C13" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E13" s="23" t="s">
         <v>22</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="H13" s="7"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="D14" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E14" s="23" t="s">
         <v>22</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>7</v>
@@ -1361,269 +1343,267 @@
       <c r="C15" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E15" s="23" t="s">
         <v>22</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="H15" s="7"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="E16" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
+      <c r="D16" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>66</v>
+      </c>
       <c r="H16" s="7"/>
     </row>
-    <row r="17" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="7"/>
+    </row>
+    <row r="18" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B18" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C18" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="E17" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="9"/>
-    </row>
-    <row r="18" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="B19" s="4" t="s">
+      <c r="D18" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="9"/>
+    </row>
+    <row r="19" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D19" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="E19" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="F19" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="H19" s="5"/>
-    </row>
-    <row r="20" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="B20" s="8" t="s">
+      <c r="D20" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="H20" s="5"/>
+    </row>
+    <row r="21" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D20" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="E20" s="8" t="s">
+      <c r="C21" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="F20" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="H20" s="9"/>
-    </row>
-    <row r="21" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
+      <c r="D21" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="H21" s="9"/>
+    </row>
+    <row r="22" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B23" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C23" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D22" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="5"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="20" t="s">
-        <v>110</v>
-      </c>
-      <c r="B23" s="2" t="s">
+      <c r="D23" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="E23" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D23" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="E23" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="G23" s="2"/>
-      <c r="H23" s="22"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D24" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E24" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>108</v>
-      </c>
+      <c r="D24" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G24" s="2"/>
+      <c r="H24" s="22"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D25" s="17" t="s">
-        <v>86</v>
+      <c r="D25" s="15" t="s">
+        <v>22</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
+        <v>60</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>94</v>
+      </c>
       <c r="H25" s="7" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D26" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H26" s="7"/>
+        <v>21</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E26" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="7" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="6" t="s">
-        <v>64</v>
+        <v>30</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D27" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H27" s="7"/>
+        <v>21</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="7" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
-        <v>63</v>
+        <v>110</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>12</v>
@@ -1631,23 +1611,25 @@
       <c r="C28" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D28" s="23" t="s">
+      <c r="D28" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H28" s="7"/>
+        <v>72</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="6" t="s">
-        <v>57</v>
+        <v>111</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>12</v>
@@ -1655,177 +1637,177 @@
       <c r="C29" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D29" s="23" t="s">
+      <c r="D29" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="H29" s="7"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B30" s="1" t="s">
+    <row r="30" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="B30" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D30" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H30" s="7"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D31" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H31" s="7"/>
+      <c r="D30" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="H30" s="9"/>
+    </row>
+    <row r="31" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="10"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="10"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D32" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H32" s="7"/>
+      <c r="A32" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D32" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="E32" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="H32" s="5"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="6" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D33" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>68</v>
+        <v>32</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E33" s="23" t="s">
+        <v>22</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>85</v>
+        <v>34</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>100</v>
       </c>
       <c r="H33" s="7"/>
     </row>
-    <row r="34" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="11" t="s">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E34" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H34" s="7"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E35" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G35" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="D34" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="G34" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="H34" s="9"/>
-    </row>
-    <row r="35" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="10"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="27"/>
-      <c r="H35" s="10"/>
+      <c r="H35" s="7"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C36" s="4" t="s">
+      <c r="A36" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D36" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="E36" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="G36" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="H36" s="5"/>
+      <c r="D36" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E36" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H36" s="7"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" s="6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>12</v>
@@ -1833,162 +1815,66 @@
       <c r="C37" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D37" s="23" t="s">
+      <c r="D37" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E37" s="23" t="s">
         <v>22</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G37" s="10" t="s">
-        <v>113</v>
+        <v>43</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>101</v>
       </c>
       <c r="H37" s="7"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B38" s="1" t="s">
+    <row r="38" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B38" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D38" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E38" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="H38" s="7"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D39" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E39" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="H39" s="7"/>
+      <c r="D38" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="E38" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G38" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="H38" s="9"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D40" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E40" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H40" s="7"/>
+      <c r="A40" t="s">
+        <v>107</v>
+      </c>
+      <c r="B40" t="s">
+        <v>102</v>
+      </c>
+      <c r="C40" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D41" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E41" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="H41" s="7"/>
-    </row>
-    <row r="42" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B42" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C42" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D42" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="E42" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="F42" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="G42" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="H42" s="9"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>120</v>
-      </c>
-      <c r="B44" t="s">
-        <v>115</v>
-      </c>
-      <c r="C44" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>117</v>
-      </c>
-      <c r="B45" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>119</v>
+      <c r="A41" t="s">
+        <v>104</v>
+      </c>
+      <c r="B41" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -2028,19 +1914,19 @@
         <v>28</v>
       </c>
       <c r="G1" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="H1" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="I1" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="J1" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="K1" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
@@ -2048,31 +1934,31 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="C2" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="D2" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="E2" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="F2" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="G2" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="H2" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="I2" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="J2" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="K2">
         <v>8</v>
@@ -2083,31 +1969,31 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="C3" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="D3" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="E3" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="F3" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="G3" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="H3" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="I3" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="J3" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="K3">
         <v>1</v>
@@ -2118,31 +2004,31 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="E4" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="F4" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="G4" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="H4" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="I4" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="J4" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="K4">
         <v>1</v>
@@ -2153,31 +2039,31 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="E5" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="F5" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="G5" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="H5" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="I5" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="J5" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="K5">
         <v>2</v>
@@ -2188,31 +2074,31 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="C6" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="D6" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="E6" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="F6" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="G6" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="H6" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="I6" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="J6" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="K6">
         <v>3</v>
@@ -2223,31 +2109,31 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="E7" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="F7" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="G7" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="H7" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="I7" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="J7" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="K7">
         <v>20</v>
@@ -2258,31 +2144,31 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="C8" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="D8" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="E8" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="F8" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="G8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="H8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="I8" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="J8" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="K8">
         <v>100</v>

</xml_diff>

<commit_message>
add file for health_checks and modify features table
</commit_message>
<xml_diff>
--- a/features.xlsx
+++ b/features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakoberhard/Library/CloudStorage/GoogleDrive-jakanterh@gmail.com/My Drive/uni/python/TBA_project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D29E5851-0560-E84E-9C3A-10DD19C89B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33761C64-A4DC-E84C-B233-6FCA27BB99F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="107">
   <si>
     <t>feature</t>
   </si>
@@ -148,12 +148,6 @@
     <t>time_till_dest_planned</t>
   </si>
   <si>
-    <t>arrival_current_station - depature_first_station</t>
-  </si>
-  <si>
-    <t>arrival_last_station - depature_current_station</t>
-  </si>
-  <si>
     <t>station_role</t>
   </si>
   <si>
@@ -232,18 +226,6 @@
     <t>availability api data</t>
   </si>
   <si>
-    <t>route_related_history</t>
-  </si>
-  <si>
-    <t>hist_delay_avg_route</t>
-  </si>
-  <si>
-    <t>hist_delay_sd_route</t>
-  </si>
-  <si>
-    <t>group all connections that have common start station and current station (trains coming from X, how much delay do they have at Y?)</t>
-  </si>
-  <si>
     <t>from historical data (saved from training)</t>
   </si>
   <si>
@@ -289,21 +271,12 @@
     <t>Halt 5</t>
   </si>
   <si>
-    <t>arrival_planned</t>
-  </si>
-  <si>
     <t>arrival_real</t>
   </si>
   <si>
     <t>NA</t>
   </si>
   <si>
-    <t>depature_planned</t>
-  </si>
-  <si>
-    <t>depature_real</t>
-  </si>
-  <si>
     <t>ZEIT</t>
   </si>
   <si>
@@ -319,9 +292,6 @@
     <t>we can leave the weather for every station out, this would reduce complexity because we then only have 2 weather api calls for every train ride</t>
   </si>
   <si>
-    <t>time_current_planned</t>
-  </si>
-  <si>
     <t>planned_depature</t>
   </si>
   <si>
@@ -334,24 +304,6 @@
     <t>above needed</t>
   </si>
   <si>
-    <t>actual delays</t>
-  </si>
-  <si>
-    <t>same day delay on station</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stationen außerhalb deutschland </t>
-  </si>
-  <si>
-    <t>NA für bestimmte variablen (stops etc.)</t>
-  </si>
-  <si>
-    <t>modell fertigstellen</t>
-  </si>
-  <si>
-    <t>eventuell feature bauen</t>
-  </si>
-  <si>
     <t>hour</t>
   </si>
   <si>
@@ -374,6 +326,27 @@
   </si>
   <si>
     <t>canceled</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>time_current_arrival_planned</t>
+  </si>
+  <si>
+    <t>time_current_departure_planned</t>
+  </si>
+  <si>
+    <t>time_current__departure_real</t>
+  </si>
+  <si>
+    <t>time_current_departure_real</t>
+  </si>
+  <si>
+    <t>arrival_current_station - departure_first_station</t>
+  </si>
+  <si>
+    <t>arrival_last_station - departure_current_station</t>
   </si>
 </sst>
 </file>
@@ -684,7 +657,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -714,6 +687,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -994,7 +968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.6640625" bestFit="1" customWidth="1"/>
@@ -1018,19 +992,19 @@
         <v>1</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -1044,16 +1018,16 @@
         <v>20</v>
       </c>
       <c r="D2" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>57</v>
       </c>
       <c r="H2" s="5"/>
     </row>
@@ -1068,15 +1042,15 @@
         <v>20</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -1090,10 +1064,10 @@
         <v>20</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -1113,13 +1087,13 @@
         <v>22</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="H5" s="7"/>
     </row>
@@ -1134,20 +1108,20 @@
         <v>20</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="H6" s="7"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>15</v>
@@ -1156,10 +1130,10 @@
         <v>20</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -1167,7 +1141,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>12</v>
@@ -1185,7 +1159,7 @@
         <v>26</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H8" s="7"/>
     </row>
@@ -1209,7 +1183,7 @@
         <v>23</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H9" s="7"/>
     </row>
@@ -1233,7 +1207,7 @@
         <v>24</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H10" s="7"/>
     </row>
@@ -1257,7 +1231,7 @@
         <v>25</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H11" s="7"/>
     </row>
@@ -1278,10 +1252,10 @@
         <v>22</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H12" s="7"/>
     </row>
@@ -1302,10 +1276,10 @@
         <v>22</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H13" s="7"/>
     </row>
@@ -1326,10 +1300,10 @@
         <v>22</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H14" s="7"/>
     </row>
@@ -1350,10 +1324,10 @@
         <v>22</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H15" s="7"/>
     </row>
@@ -1374,10 +1348,10 @@
         <v>22</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H16" s="7"/>
     </row>
@@ -1392,10 +1366,10 @@
         <v>20</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
@@ -1412,10 +1386,10 @@
         <v>20</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F18" s="8"/>
       <c r="G18" s="8"/>
@@ -1433,110 +1407,118 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
-        <v>69</v>
+        <v>28</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D20" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>72</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
       <c r="H20" s="5"/>
     </row>
-    <row r="21" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="D21" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="G21" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="H21" s="9"/>
-    </row>
-    <row r="22" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="H21" s="22"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="E22" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="22"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C23" s="4" t="s">
+      <c r="A23" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D23" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="E23" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="5"/>
+      <c r="D23" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="E23" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="22"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C24" s="2" t="s">
+      <c r="A24" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D24" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="E24" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="G24" s="2"/>
-      <c r="H24" s="22"/>
+      <c r="D24" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
-        <v>29</v>
+        <v>92</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>21</v>
@@ -1544,174 +1526,172 @@
       <c r="D25" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>94</v>
-      </c>
+      <c r="E25" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
       <c r="H25" s="7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
-        <v>108</v>
+        <v>30</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D26" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E26" s="23" t="s">
-        <v>22</v>
+      <c r="D26" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>67</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="7" t="s">
-        <v>109</v>
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="6" t="s">
-        <v>30</v>
+        <v>94</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D27" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="E27" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
+        <v>48</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>66</v>
+      </c>
       <c r="H27" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H28" s="7"/>
+    </row>
+    <row r="29" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D29" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F29" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D28" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H28" s="7" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="B29" s="1" t="s">
+      <c r="G29" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="H29" s="9"/>
+    </row>
+    <row r="30" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="10"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="10"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="E31" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="H31" s="5"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D29" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H29" s="7"/>
-    </row>
-    <row r="30" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="D30" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="G30" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="H30" s="9"/>
-    </row>
-    <row r="31" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="10"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="E32" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="G32" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="H32" s="5"/>
+      <c r="D32" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E32" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="H32" s="7"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="6" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>12</v>
@@ -1726,19 +1706,19 @@
         <v>22</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G33" s="10" t="s">
-        <v>100</v>
+        <v>45</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H33" s="7"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>32</v>
@@ -1750,16 +1730,16 @@
         <v>22</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>47</v>
+        <v>105</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H34" s="7"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>14</v>
@@ -1774,19 +1754,19 @@
         <v>22</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>40</v>
+        <v>106</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H35" s="7"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>32</v>
@@ -1801,81 +1781,33 @@
         <v>41</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="H36" s="7"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" s="6" t="s">
+    <row r="37" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D37" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="E37" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F37" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B37" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D37" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E37" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="H37" s="7"/>
-    </row>
-    <row r="38" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C38" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D38" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="E38" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="F38" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="G38" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="H38" s="9"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>107</v>
-      </c>
-      <c r="B40" t="s">
-        <v>102</v>
-      </c>
-      <c r="C40" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>104</v>
-      </c>
-      <c r="B41" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>106</v>
-      </c>
+      <c r="G37" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="H37" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1884,28 +1816,29 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E59CFC8-413C-463C-B177-BDA848B5E119}">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" customWidth="1"/>
     <col min="5" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.6640625" customWidth="1"/>
+    <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>4</v>
-      </c>
-      <c r="D1" t="s">
-        <v>5</v>
       </c>
       <c r="E1" t="s">
         <v>37</v>
@@ -1914,263 +1847,287 @@
         <v>28</v>
       </c>
       <c r="G1" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="H1" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="I1" t="s">
-        <v>90</v>
-      </c>
-      <c r="J1" t="s">
-        <v>91</v>
+        <v>81</v>
+      </c>
+      <c r="J1" s="29" t="s">
+        <v>102</v>
       </c>
       <c r="K1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+        <v>103</v>
+      </c>
+      <c r="L1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>82</v>
+      </c>
+      <c r="I2" t="s">
+        <v>82</v>
+      </c>
+      <c r="J2" t="s">
+        <v>83</v>
+      </c>
+      <c r="K2" t="s">
+        <v>83</v>
+      </c>
+      <c r="L2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F3" t="s">
+        <v>76</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>83</v>
+      </c>
+      <c r="I3" t="s">
+        <v>83</v>
+      </c>
+      <c r="J3" t="s">
+        <v>83</v>
+      </c>
+      <c r="K3" t="s">
+        <v>83</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s">
+        <v>83</v>
+      </c>
+      <c r="I4" t="s">
+        <v>83</v>
+      </c>
+      <c r="J4" t="s">
+        <v>83</v>
+      </c>
+      <c r="K4" t="s">
+        <v>83</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E5" t="s">
+        <v>75</v>
+      </c>
+      <c r="F5" t="s">
         <v>78</v>
       </c>
-      <c r="C2" t="s">
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="s">
+        <v>83</v>
+      </c>
+      <c r="I5" t="s">
+        <v>83</v>
+      </c>
+      <c r="J5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K5" t="s">
+        <v>83</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F6" t="s">
         <v>79</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>83</v>
+      </c>
+      <c r="I6" t="s">
+        <v>83</v>
+      </c>
+      <c r="J6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K6" t="s">
+        <v>83</v>
+      </c>
+      <c r="L6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F7" t="s">
         <v>80</v>
       </c>
-      <c r="E2" t="s">
-        <v>81</v>
-      </c>
-      <c r="F2" t="s">
-        <v>80</v>
-      </c>
-      <c r="G2" t="s">
-        <v>89</v>
-      </c>
-      <c r="H2" t="s">
-        <v>89</v>
-      </c>
-      <c r="I2" t="s">
-        <v>92</v>
-      </c>
-      <c r="J2" t="s">
-        <v>92</v>
-      </c>
-      <c r="K2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>83</v>
+      </c>
+      <c r="I7" t="s">
+        <v>83</v>
+      </c>
+      <c r="J7" t="s">
+        <v>83</v>
+      </c>
+      <c r="K7" t="s">
+        <v>83</v>
+      </c>
+      <c r="L7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C3" t="s">
-        <v>79</v>
-      </c>
-      <c r="D3" t="s">
-        <v>80</v>
-      </c>
-      <c r="E3" t="s">
-        <v>81</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="C8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" t="s">
+        <v>75</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
+        <v>83</v>
+      </c>
+      <c r="I8" t="s">
+        <v>83</v>
+      </c>
+      <c r="J8" t="s">
         <v>82</v>
       </c>
-      <c r="G3" t="s">
-        <v>92</v>
-      </c>
-      <c r="H3" t="s">
-        <v>92</v>
-      </c>
-      <c r="I3" t="s">
-        <v>92</v>
-      </c>
-      <c r="J3" t="s">
-        <v>92</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E4" t="s">
-        <v>81</v>
-      </c>
-      <c r="F4" t="s">
-        <v>83</v>
-      </c>
-      <c r="G4" t="s">
-        <v>92</v>
-      </c>
-      <c r="H4" t="s">
-        <v>92</v>
-      </c>
-      <c r="I4" t="s">
-        <v>92</v>
-      </c>
-      <c r="J4" t="s">
-        <v>92</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C5" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" t="s">
-        <v>80</v>
-      </c>
-      <c r="E5" t="s">
-        <v>81</v>
-      </c>
-      <c r="F5" t="s">
-        <v>84</v>
-      </c>
-      <c r="G5" t="s">
-        <v>92</v>
-      </c>
-      <c r="H5" t="s">
-        <v>92</v>
-      </c>
-      <c r="I5" t="s">
-        <v>92</v>
-      </c>
-      <c r="J5" t="s">
-        <v>92</v>
-      </c>
-      <c r="K5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>1</v>
-      </c>
-      <c r="B6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C6" t="s">
-        <v>79</v>
-      </c>
-      <c r="D6" t="s">
-        <v>80</v>
-      </c>
-      <c r="E6" t="s">
-        <v>81</v>
-      </c>
-      <c r="F6" t="s">
-        <v>85</v>
-      </c>
-      <c r="G6" t="s">
-        <v>92</v>
-      </c>
-      <c r="H6" t="s">
-        <v>92</v>
-      </c>
-      <c r="I6" t="s">
-        <v>92</v>
-      </c>
-      <c r="J6" t="s">
-        <v>92</v>
-      </c>
-      <c r="K6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="B7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C7" t="s">
-        <v>79</v>
-      </c>
-      <c r="D7" t="s">
-        <v>80</v>
-      </c>
-      <c r="E7" t="s">
-        <v>81</v>
-      </c>
-      <c r="F7" t="s">
-        <v>86</v>
-      </c>
-      <c r="G7" t="s">
-        <v>92</v>
-      </c>
-      <c r="H7" t="s">
-        <v>92</v>
-      </c>
-      <c r="I7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J7" t="s">
-        <v>92</v>
-      </c>
-      <c r="K7">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>1</v>
-      </c>
-      <c r="B8" t="s">
-        <v>78</v>
-      </c>
-      <c r="C8" t="s">
-        <v>79</v>
-      </c>
-      <c r="D8" t="s">
-        <v>80</v>
-      </c>
-      <c r="E8" t="s">
-        <v>81</v>
-      </c>
-      <c r="F8" t="s">
-        <v>81</v>
-      </c>
-      <c r="G8" t="s">
-        <v>92</v>
-      </c>
-      <c r="H8" t="s">
-        <v>92</v>
-      </c>
-      <c r="I8" t="s">
-        <v>89</v>
-      </c>
-      <c r="J8" t="s">
-        <v>89</v>
-      </c>
-      <c r="K8">
+      <c r="K8" t="s">
+        <v>82</v>
+      </c>
+      <c r="L8">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
write data wrangling function
</commit_message>
<xml_diff>
--- a/features.xlsx
+++ b/features.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10201"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakoberhard/Library/CloudStorage/GoogleDrive-jakanterh@gmail.com/My Drive/uni/python/TBA_project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33761C64-A4DC-E84C-B233-6FCA27BB99F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866C2C2E-F4D3-754A-B578-497F3D14ABCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="features" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="98">
   <si>
     <t>feature</t>
   </si>
@@ -46,9 +46,6 @@
     <t>station_start</t>
   </si>
   <si>
-    <t>time_start_planned</t>
-  </si>
-  <si>
     <t>category</t>
   </si>
   <si>
@@ -58,9 +55,6 @@
     <t>weekday</t>
   </si>
   <si>
-    <t>weekend</t>
-  </si>
-  <si>
     <t>pandas data_type</t>
   </si>
   <si>
@@ -82,12 +76,6 @@
     <t>month</t>
   </si>
   <si>
-    <t>season</t>
-  </si>
-  <si>
-    <t>weather_start</t>
-  </si>
-  <si>
     <t>ride_related</t>
   </si>
   <si>
@@ -118,36 +106,21 @@
     <t>dwell_time_planned</t>
   </si>
   <si>
-    <t>weather_current</t>
-  </si>
-  <si>
     <t xml:space="preserve">planned_depature - planned_arrival </t>
   </si>
   <si>
     <t>sequence_related</t>
   </si>
   <si>
-    <t>stops_remaining</t>
-  </si>
-  <si>
     <t>row number grouped by unique ride</t>
   </si>
   <si>
     <t>time_since_start_planned</t>
   </si>
   <si>
-    <t>time_dest_planned</t>
-  </si>
-  <si>
     <t>station_dest</t>
   </si>
   <si>
-    <t>weather_dest</t>
-  </si>
-  <si>
-    <t>time_till_dest_planned</t>
-  </si>
-  <si>
     <t>station_role</t>
   </si>
   <si>
@@ -157,15 +130,6 @@
     <t>share_ride_time</t>
   </si>
   <si>
-    <t>share_ride_stations</t>
-  </si>
-  <si>
-    <t>stops_index / stops_total</t>
-  </si>
-  <si>
-    <t>stops_total - stops_index - 1</t>
-  </si>
-  <si>
     <t>stops_index</t>
   </si>
   <si>
@@ -178,9 +142,6 @@
     <t>see above only for specific day</t>
   </si>
   <si>
-    <t>see above only for specific hour</t>
-  </si>
-  <si>
     <t>start / stopover / destination</t>
   </si>
   <si>
@@ -340,13 +301,25 @@
     <t>time_current__departure_real</t>
   </si>
   <si>
-    <t>time_current_departure_real</t>
-  </si>
-  <si>
     <t>arrival_current_station - departure_first_station</t>
   </si>
   <si>
-    <t>arrival_last_station - departure_current_station</t>
+    <t>departure_planned</t>
+  </si>
+  <si>
+    <t>arrival_planned</t>
+  </si>
+  <si>
+    <t>departure_planned_start</t>
+  </si>
+  <si>
+    <t>arrival_planned_dest</t>
+  </si>
+  <si>
+    <t>weather</t>
+  </si>
+  <si>
+    <t>group by station/hour and give delay (mean/sd/q90/count)</t>
   </si>
 </sst>
 </file>
@@ -657,7 +630,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -687,7 +660,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -968,7 +940,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.6640625" bestFit="1" customWidth="1"/>
@@ -986,25 +958,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="13" t="s">
-        <v>65</v>
-      </c>
       <c r="F1" s="13" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -1012,22 +984,22 @@
         <v>2</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="H2" s="5"/>
     </row>
@@ -1036,21 +1008,21 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="7" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -1058,16 +1030,16 @@
         <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -1078,136 +1050,140 @@
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="H5" s="7"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="H6" s="7"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>99</v>
+        <v>35</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="E7" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
+        <v>18</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>6</v>
+        <v>95</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="G9" s="1" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H9" s="7"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="H10" s="7"/>
     </row>
@@ -1216,598 +1192,414 @@
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="H11" s="7"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="H12" s="7"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H13" s="7"/>
+    </row>
+    <row r="14" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E13" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H13" s="7"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="6" t="s">
+      <c r="C14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E14" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H14" s="7"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="6" t="s">
+      <c r="D14" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="9"/>
+    </row>
+    <row r="15" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E15" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H15" s="7"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E16" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H16" s="7"/>
+      <c r="D16" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="5"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="1" t="s">
+      <c r="A17" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G17" s="2"/>
+      <c r="H17" s="22"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="E18" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="22"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D17" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="E17" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="7"/>
-    </row>
-    <row r="18" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
+      <c r="C19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H23" s="7"/>
+    </row>
+    <row r="24" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D24" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H24" s="9"/>
+    </row>
+    <row r="25" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="10"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="E26" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="9"/>
-    </row>
-    <row r="19" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D20" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="E20" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="5"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="20" t="s">
-        <v>102</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="E21" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="G21" s="2"/>
-      <c r="H21" s="22"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="20" t="s">
-        <v>104</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="E22" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="22"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="E23" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="22"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E24" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D25" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E25" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="7" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D26" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="E26" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="7" t="s">
-        <v>87</v>
-      </c>
+      <c r="G26" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="H26" s="5"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="6" t="s">
-        <v>94</v>
+        <v>34</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>54</v>
+        <v>18</v>
+      </c>
+      <c r="E27" s="23" t="s">
+        <v>18</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>98</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="G27" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="H27" s="7"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
-        <v>95</v>
+        <v>29</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>54</v>
+        <v>18</v>
+      </c>
+      <c r="E28" s="23" t="s">
+        <v>18</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>49</v>
+        <v>91</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="H28" s="7"/>
     </row>
     <row r="29" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>96</v>
+        <v>33</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>54</v>
+        <v>18</v>
+      </c>
+      <c r="E29" s="25" t="s">
+        <v>18</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="H29" s="9"/>
-    </row>
-    <row r="30" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="10"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="10"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D31" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="E31" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="G31" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="H31" s="5"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D32" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E32" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G32" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="H32" s="7"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E33" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="H33" s="7"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D34" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E34" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="H34" s="7"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D35" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E35" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H35" s="7"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D36" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E36" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H36" s="7"/>
-    </row>
-    <row r="37" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C37" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D37" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="E37" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="F37" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G37" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="H37" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1829,7 +1621,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>
@@ -1841,28 +1633,28 @@
         <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G1" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="H1" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="I1" t="s">
-        <v>81</v>
-      </c>
-      <c r="J1" s="29" t="s">
-        <v>102</v>
+        <v>68</v>
+      </c>
+      <c r="J1" t="s">
+        <v>89</v>
       </c>
       <c r="K1" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="L1" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
@@ -1873,31 +1665,31 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="F2" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="I2" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="J2" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="K2" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="L2">
         <v>8</v>
@@ -1911,31 +1703,31 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E3" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="F3" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="I3" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="J3" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="K3" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="L3">
         <v>1</v>
@@ -1949,31 +1741,31 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E4" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="I4" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="J4" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="K4" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="L4">
         <v>1</v>
@@ -1987,31 +1779,31 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E5" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="F5" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="I5" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="J5" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="K5" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="L5">
         <v>2</v>
@@ -2025,31 +1817,31 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="I6" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="J6" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="K6" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="L6">
         <v>3</v>
@@ -2063,31 +1855,31 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E7" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="F7" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="I7" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="J7" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="K7" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="L7">
         <v>20</v>
@@ -2101,31 +1893,31 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E8" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="I8" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="J8" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="K8" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="L8">
         <v>100</v>

</xml_diff>